<commit_message>
chore: add OCR capture brief + scan output artifacts, local settings
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/output/medias-manquants.xlsx
+++ b/scripts/output/medias-manquants.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vgail\Documents\projets\eatSafe\scripts\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92103333-B018-4161-98B5-2ED396CEFD53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{956D1BDF-2358-4FFA-AF51-BD1FE57D5926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Médias manquants" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -740,7 +741,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -750,6 +751,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -766,9 +773,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2100,7 +2108,7 @@
       <c r="D58" t="s">
         <v>124</v>
       </c>
-      <c r="E58" t="s">
+      <c r="E58" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2117,7 +2125,7 @@
       <c r="D59" t="s">
         <v>126</v>
       </c>
-      <c r="E59" t="s">
+      <c r="E59" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2134,7 +2142,7 @@
       <c r="D60" t="s">
         <v>128</v>
       </c>
-      <c r="E60" t="s">
+      <c r="E60" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2151,7 +2159,7 @@
       <c r="D61" t="s">
         <v>130</v>
       </c>
-      <c r="E61" t="s">
+      <c r="E61" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2168,7 +2176,7 @@
       <c r="D62" t="s">
         <v>132</v>
       </c>
-      <c r="E62" t="s">
+      <c r="E62" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2185,7 +2193,7 @@
       <c r="D63" t="s">
         <v>134</v>
       </c>
-      <c r="E63" t="s">
+      <c r="E63" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2202,7 +2210,7 @@
       <c r="D64" t="s">
         <v>136</v>
       </c>
-      <c r="E64" t="s">
+      <c r="E64" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2219,7 +2227,7 @@
       <c r="D65" t="s">
         <v>138</v>
       </c>
-      <c r="E65" t="s">
+      <c r="E65" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2236,7 +2244,7 @@
       <c r="D66" t="s">
         <v>140</v>
       </c>
-      <c r="E66" t="s">
+      <c r="E66" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2253,7 +2261,7 @@
       <c r="D67" t="s">
         <v>142</v>
       </c>
-      <c r="E67" t="s">
+      <c r="E67" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2270,7 +2278,7 @@
       <c r="D68" t="s">
         <v>144</v>
       </c>
-      <c r="E68" t="s">
+      <c r="E68" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2287,7 +2295,7 @@
       <c r="D69" t="s">
         <v>146</v>
       </c>
-      <c r="E69" t="s">
+      <c r="E69" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2304,7 +2312,7 @@
       <c r="D70" t="s">
         <v>148</v>
       </c>
-      <c r="E70" t="s">
+      <c r="E70" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2321,7 +2329,7 @@
       <c r="D71" t="s">
         <v>150</v>
       </c>
-      <c r="E71" t="s">
+      <c r="E71" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2338,7 +2346,7 @@
       <c r="D72" t="s">
         <v>152</v>
       </c>
-      <c r="E72" t="s">
+      <c r="E72" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2355,7 +2363,7 @@
       <c r="D73" t="s">
         <v>154</v>
       </c>
-      <c r="E73" t="s">
+      <c r="E73" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2372,7 +2380,7 @@
       <c r="D74" t="s">
         <v>156</v>
       </c>
-      <c r="E74" t="s">
+      <c r="E74" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2389,7 +2397,7 @@
       <c r="D75" t="s">
         <v>158</v>
       </c>
-      <c r="E75" t="s">
+      <c r="E75" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2406,7 +2414,7 @@
       <c r="D76" t="s">
         <v>160</v>
       </c>
-      <c r="E76" t="s">
+      <c r="E76" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2423,7 +2431,7 @@
       <c r="D77" t="s">
         <v>162</v>
       </c>
-      <c r="E77" t="s">
+      <c r="E77" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2440,7 +2448,7 @@
       <c r="D78" t="s">
         <v>164</v>
       </c>
-      <c r="E78" t="s">
+      <c r="E78" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2457,7 +2465,7 @@
       <c r="D79" t="s">
         <v>166</v>
       </c>
-      <c r="E79" t="s">
+      <c r="E79" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2474,7 +2482,7 @@
       <c r="D80" t="s">
         <v>168</v>
       </c>
-      <c r="E80" t="s">
+      <c r="E80" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2491,7 +2499,7 @@
       <c r="D81" t="s">
         <v>170</v>
       </c>
-      <c r="E81" t="s">
+      <c r="E81" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2508,7 +2516,7 @@
       <c r="D82" t="s">
         <v>172</v>
       </c>
-      <c r="E82" t="s">
+      <c r="E82" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2525,7 +2533,7 @@
       <c r="D83" t="s">
         <v>174</v>
       </c>
-      <c r="E83" t="s">
+      <c r="E83" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2542,7 +2550,7 @@
       <c r="D84" t="s">
         <v>176</v>
       </c>
-      <c r="E84" t="s">
+      <c r="E84" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2559,7 +2567,7 @@
       <c r="D85" t="s">
         <v>178</v>
       </c>
-      <c r="E85" t="s">
+      <c r="E85" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2576,7 +2584,7 @@
       <c r="D86" t="s">
         <v>180</v>
       </c>
-      <c r="E86" t="s">
+      <c r="E86" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2593,7 +2601,7 @@
       <c r="D87" t="s">
         <v>183</v>
       </c>
-      <c r="E87" t="s">
+      <c r="E87" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2610,7 +2618,7 @@
       <c r="D88" t="s">
         <v>185</v>
       </c>
-      <c r="E88" t="s">
+      <c r="E88" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2627,7 +2635,7 @@
       <c r="D89" t="s">
         <v>187</v>
       </c>
-      <c r="E89" t="s">
+      <c r="E89" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2644,7 +2652,7 @@
       <c r="D90" t="s">
         <v>189</v>
       </c>
-      <c r="E90" t="s">
+      <c r="E90" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2661,7 +2669,7 @@
       <c r="D91" t="s">
         <v>191</v>
       </c>
-      <c r="E91" t="s">
+      <c r="E91" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2678,7 +2686,7 @@
       <c r="D92" t="s">
         <v>193</v>
       </c>
-      <c r="E92" t="s">
+      <c r="E92" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2695,7 +2703,7 @@
       <c r="D93" t="s">
         <v>195</v>
       </c>
-      <c r="E93" t="s">
+      <c r="E93" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2712,7 +2720,7 @@
       <c r="D94" t="s">
         <v>197</v>
       </c>
-      <c r="E94" t="s">
+      <c r="E94" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2729,7 +2737,7 @@
       <c r="D95" t="s">
         <v>199</v>
       </c>
-      <c r="E95" t="s">
+      <c r="E95" s="1" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>